<commit_message>
feat: favicon EMS Dev + nettoyage fichiers obsoletes + devops-manager updates
</commit_message>
<xml_diff>
--- a/TEMPLATE_IMPORT_EMPLOYES_EMS_v2.xlsx
+++ b/TEMPLATE_IMPORT_EMPLOYES_EMS_v2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cedri\OneDrive - ELITE CAPITAL Group S.A\Documents\EMS\extranet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{699116ED-D3D8-4819-9758-B0CC3C03E508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0C479EF-8F20-481D-948B-EFD25713FB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -932,10 +932,10 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -9931,7 +9931,7 @@
       <c r="A27" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="B27" s="19" t="s">
+      <c r="B27" s="20" t="s">
         <v>105</v>
       </c>
       <c r="C27" s="15"/>
@@ -9943,7 +9943,7 @@
       <c r="A28" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="B28" s="20" t="s">
+      <c r="B28" s="19" t="s">
         <v>106</v>
       </c>
       <c r="C28" s="15"/>
@@ -9967,7 +9967,7 @@
       <c r="A30" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B30" s="20" t="s">
+      <c r="B30" s="19" t="s">
         <v>108</v>
       </c>
       <c r="C30" s="15"/>
@@ -9991,7 +9991,7 @@
       <c r="A32" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B32" s="20" t="s">
+      <c r="B32" s="19" t="s">
         <v>110</v>
       </c>
       <c r="C32" s="15"/>
@@ -10089,6 +10089,10 @@
     <mergeCell ref="B32:F32"/>
     <mergeCell ref="B35:F35"/>
     <mergeCell ref="A34:F34"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B7:F7"/>
     <mergeCell ref="B40:F40"/>
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B30:F30"/>
@@ -10096,7 +10100,6 @@
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B15:F15"/>
-    <mergeCell ref="A3:F3"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B21:F21"/>
@@ -10106,14 +10109,11 @@
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B29:F29"/>
     <mergeCell ref="B38:F38"/>
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B37:F37"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B7:F7"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B31:F31"/>
     <mergeCell ref="A12:F12"/>

</xml_diff>